<commit_message>
add batch of problem solutions
</commit_message>
<xml_diff>
--- a/Practice Coding 1/Docs/Class DSA Pattern Questions Tracker.xlsx
+++ b/Practice Coding 1/Docs/Class DSA Pattern Questions Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\B.Tech\Semester 05\Practice Coding\Practice Coding 1\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E0570D9-BE09-48DB-94C4-51978A2BA617}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2518CF5E-0BE2-4A5D-91E1-BB81B1B1C554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C15" s="16">
         <f>COUNTIF(Tracker!$J:$J,"Solved")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D15" s="17" t="s">
         <v>70</v>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="C19" s="16">
         <f>COUNTIFS(Tracker!$B:$B,"Homework",Tracker!$J:$J,"Solved")</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D19" s="17" t="s">
         <v>102</v>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="C20" s="16" t="str">
         <f>ROUND(COUNTIF(Tracker!$J:$J,"Solved")/480*100,1)&amp;"%"</f>
-        <v>1.9%</v>
+        <v>2.3%</v>
       </c>
       <c r="D20" s="17"/>
     </row>
@@ -8810,7 +8810,7 @@
         <v>22</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="K11" s="20"/>
     </row>
@@ -8843,7 +8843,7 @@
         <v>22</v>
       </c>
       <c r="J12" s="19" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="K12" s="20"/>
     </row>

</xml_diff>

<commit_message>
add several coding problem solutions
</commit_message>
<xml_diff>
--- a/Practice Coding 1/Docs/Class DSA Pattern Questions Tracker.xlsx
+++ b/Practice Coding 1/Docs/Class DSA Pattern Questions Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\B.Tech\Semester 05\Practice Coding\Practice Coding 1\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2518CF5E-0BE2-4A5D-91E1-BB81B1B1C554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AC4CE42-56FE-4BD3-9C4C-738772CE250D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3631,7 +3631,7 @@
       </c>
       <c r="C15" s="16">
         <f>COUNTIF(Tracker!$J:$J,"Solved")</f>
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D15" s="17" t="s">
         <v>70</v>
@@ -3663,7 +3663,7 @@
       </c>
       <c r="C18" s="16">
         <f>COUNTIFS(Tracker!$B:$B,"In-Class",Tracker!$J:$J,"Solved")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D18" s="17" t="s">
         <v>93</v>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="C19" s="16">
         <f>COUNTIFS(Tracker!$B:$B,"Homework",Tracker!$J:$J,"Solved")</f>
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D19" s="17" t="s">
         <v>102</v>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="C20" s="16" t="str">
         <f>ROUND(COUNTIF(Tracker!$J:$J,"Solved")/480*100,1)&amp;"%"</f>
-        <v>2.3%</v>
+        <v>3.5%</v>
       </c>
       <c r="D20" s="17"/>
     </row>
@@ -8876,7 +8876,7 @@
         <v>22</v>
       </c>
       <c r="J13" s="19" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="K13" s="20"/>
     </row>
@@ -8909,7 +8909,7 @@
         <v>22</v>
       </c>
       <c r="J14" s="19" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="K14" s="20"/>
     </row>
@@ -8942,7 +8942,7 @@
         <v>22</v>
       </c>
       <c r="J15" s="19" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="K15" s="20"/>
     </row>
@@ -8975,7 +8975,7 @@
         <v>22</v>
       </c>
       <c r="J16" s="19" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="K16" s="20"/>
     </row>
@@ -9041,7 +9041,7 @@
         <v>36</v>
       </c>
       <c r="J18" s="19" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="K18" s="20"/>
     </row>
@@ -9074,7 +9074,7 @@
         <v>240</v>
       </c>
       <c r="J19" s="19" t="s">
-        <v>129</v>
+        <v>92</v>
       </c>
       <c r="K19" s="20"/>
     </row>

</xml_diff>